<commit_message>
Updates for ITI MHD 4-2-5 release
</commit_message>
<xml_diff>
--- a/ITI/MHD/CodeSystem-IHE.MHD.MHDIdentifierType.xlsx
+++ b/ITI/MHD/CodeSystem-IHE.MHD.MHDIdentifierType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>4.2.5-comment</t>
+    <t>4.2.5</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-16T19:25:56-05:00</t>
+    <t>2026-10-18T17:32:41-05:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>